<commit_message>
style: fix CSS compatibility and update timetable data
</commit_message>
<xml_diff>
--- a/TimeTable.xlsx
+++ b/TimeTable.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity 개발\Prof-TimeTable\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -313,12 +318,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -326,17 +331,36 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -366,22 +390,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -423,7 +462,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -455,9 +494,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -489,6 +529,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -664,366 +705,371 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="8" width="24" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
+    <row r="3" spans="1:8" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
+    <row r="4" spans="1:8" ht="148.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
+    <row r="5" spans="1:8" ht="148.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
+    <row r="6" spans="1:8" ht="82.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
+    <row r="7" spans="1:8" ht="181.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
+    <row r="8" spans="1:8" ht="214.5" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
+    <row r="9" spans="1:8" ht="165" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
+    <row r="10" spans="1:8" ht="198" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
+    <row r="11" spans="1:8" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
+    <row r="12" spans="1:8" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
+    <row r="13" spans="1:8" ht="33" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
+    <row r="14" spans="1:8" ht="33" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
+    <row r="15" spans="1:8" ht="33" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="1" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>